<commit_message>
Fix unique and upper case for all functions
</commit_message>
<xml_diff>
--- a/static_datas/Stock_data.xlsx
+++ b/static_datas/Stock_data.xlsx
@@ -5,17 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cavidan\OneDrive\İş masası\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cavidan\JetBrainsProjects\hok-pm\server\static_datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1B1A69-F881-4AB6-AA0F-81D59D6845AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487B3BAF-7663-4C1A-8241-FF5A0E28D777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1</definedName>
+  </definedNames>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -6051,4688 +6054,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="468">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -60817,6 +56139,7 @@
       <c r="M1417" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>